<commit_message>
Fill real links: Sheets copies, Gumroad, support email
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/products/seller-profit-tracker/dist/MarginKite-Etsy-Fee-Calculator-Lite-BLANK.xlsx
+++ b/products/seller-profit-tracker/dist/MarginKite-Etsy-Fee-Calculator-Lite-BLANK.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,8 +54,13 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000563C1"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -75,11 +80,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -130,7 +130,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -734,7 +734,7 @@
     <row r="24">
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>[PLACEHOLDER: link to the full tracker goes here before launch]</t>
+          <t>Get the full tracker: marginkite.gumroad.com/l/profit-tracker</t>
         </is>
       </c>
     </row>
@@ -991,6 +991,9 @@
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>